<commit_message>
reporting and sync functionality docs
</commit_message>
<xml_diff>
--- a/bom/BOM_SpatialForagingModule.xlsx
+++ b/bom/BOM_SpatialForagingModule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mattgaidica/Documents/Software/SpatialForagingPlatform/bom/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\NeurotechHub\Programming\SpatialForagingPlatform-ProjectManager\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5371B4B6-A8E3-A240-8E89-E2ED1B89B8BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3660" yWindow="1880" windowWidth="26580" windowHeight="17760" xr2:uid="{18EBE842-4B11-444E-A9D9-2818638CA39F}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{18EBE842-4B11-444E-A9D9-2818638CA39F}"/>
   </bookViews>
   <sheets>
     <sheet name="Hardware" sheetId="1" r:id="rId1"/>
@@ -703,17 +703,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{421C52AF-D934-5E4D-A590-21C8983DA813}">
   <dimension ref="A1:K17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.83203125" style="6"/>
-    <col min="7" max="7" width="13.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="59.33203125" customWidth="1"/>
-    <col min="11" max="11" width="38.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.796875" style="6"/>
+    <col min="7" max="7" width="13.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="59.296875" customWidth="1"/>
+    <col min="11" max="11" width="38.796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -722,7 +722,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -757,7 +757,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -796,7 +796,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>38</v>
       </c>
@@ -835,7 +835,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -874,7 +874,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>72</v>
       </c>
@@ -910,7 +910,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -949,7 +949,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
@@ -988,7 +988,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>15</v>
       </c>
@@ -1027,7 +1027,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1066,7 +1066,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>19</v>
       </c>
@@ -1105,7 +1105,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>33</v>
       </c>
@@ -1144,7 +1144,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>48</v>
       </c>
@@ -1180,7 +1180,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="G16" s="5" t="s">
         <v>36</v>
       </c>
@@ -1189,7 +1189,7 @@
         <v>273.95999999999998</v>
       </c>
     </row>
-    <row r="17" spans="7:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
       <c r="G17" s="5" t="s">
         <v>37</v>
       </c>
@@ -1206,19 +1206,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8A2C5A5-03CA-4DB8-9D15-15879A9BBD02}">
   <dimension ref="A1:H14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.83203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="2"/>
-    <col min="4" max="4" width="8.83203125" style="12"/>
-    <col min="5" max="5" width="9.33203125" style="13" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.1640625" style="2" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="18.6640625" customWidth="1"/>
+    <col min="1" max="1" width="15.69921875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.796875" style="2"/>
+    <col min="4" max="4" width="8.796875" style="12"/>
+    <col min="5" max="5" width="9.296875" style="13" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.19921875" style="2" customWidth="1"/>
+    <col min="7" max="7" width="26.796875" customWidth="1"/>
+    <col min="8" max="8" width="18.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -1228,7 +1228,7 @@
       <c r="D1" s="1"/>
       <c r="E1" s="7"/>
     </row>
-    <row r="2" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2"/>
       <c r="B2"/>
       <c r="C2" s="2"/>
@@ -1236,7 +1236,7 @@
       <c r="E2" s="13"/>
       <c r="F2" s="3"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
@@ -1262,7 +1262,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>51</v>
       </c>
@@ -1286,7 +1286,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -1309,7 +1309,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>53</v>
       </c>
@@ -1333,7 +1333,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -1357,7 +1357,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>68</v>
       </c>
@@ -1403,7 +1403,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>64</v>
       </c>
@@ -1426,7 +1426,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>60</v>
       </c>
@@ -1448,7 +1448,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>61</v>
       </c>
@@ -1470,7 +1470,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>62</v>
       </c>
@@ -1495,7 +1495,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>66</v>
       </c>

</xml_diff>

<commit_message>
updates till week of 21st Sep
</commit_message>
<xml_diff>
--- a/bom/BOM_SpatialForagingModule.xlsx
+++ b/bom/BOM_SpatialForagingModule.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\NeurotechHub\Programming\SpatialForagingPlatform-ProjectManager\bom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E21470DA-0A11-44B1-9053-1086E916C8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE03F655-2BC4-4689-8A70-E23DC536C569}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{18EBE842-4B11-444E-A9D9-2818638CA39F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{18EBE842-4B11-444E-A9D9-2818638CA39F}"/>
   </bookViews>
   <sheets>
-    <sheet name="Hardware" sheetId="1" r:id="rId1"/>
-    <sheet name="Electronics" sheetId="2" r:id="rId2"/>
+    <sheet name="Electronics" sheetId="2" r:id="rId1"/>
+    <sheet name="Hardware" sheetId="1" r:id="rId2"/>
+    <sheet name="Behavior Box" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="94">
   <si>
     <t>Item</t>
   </si>
@@ -277,6 +278,51 @@
   </si>
   <si>
     <t>https://a.co/d/0hCpHv8v</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/products/47065t101/</t>
+  </si>
+  <si>
+    <t>47065t101</t>
+  </si>
+  <si>
+    <t>In future willl replace with alternative option with tapped center and 1 1/2 ft length</t>
+  </si>
+  <si>
+    <t>3 ft. T-Slot</t>
+  </si>
+  <si>
+    <t>https://www.mcmaster.com/92210A537/</t>
+  </si>
+  <si>
+    <t>1/4"-20 flat head</t>
+  </si>
+  <si>
+    <t>92210A537</t>
+  </si>
+  <si>
+    <t>https://www.tapplastics.com/product/plastics/cut_to_size_plastic/acrylic_sheets_clear/508</t>
+  </si>
+  <si>
+    <t>Clear Acrylic</t>
+  </si>
+  <si>
+    <t>https://www.tapplastics.com/product/plastics/cut_to_size_plastic/acrylic_sheets_color/341</t>
+  </si>
+  <si>
+    <t>6mm 630x400</t>
+  </si>
+  <si>
+    <t>6mm 420x420</t>
+  </si>
+  <si>
+    <t>White Acrylic</t>
+  </si>
+  <si>
+    <t>Req. pcs</t>
+  </si>
+  <si>
+    <t>Total</t>
   </si>
 </sst>
 </file>
@@ -334,7 +380,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -344,6 +390,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -362,7 +414,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
@@ -380,6 +432,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -715,509 +769,6 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{421C52AF-D934-5E4D-A590-21C8983DA813}">
-  <dimension ref="A1:K17"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="11.69921875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.796875" style="6"/>
-    <col min="7" max="7" width="13.296875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="59.296875" customWidth="1"/>
-    <col min="11" max="11" width="38.796875" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="7" t="s">
-        <v>4</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
-      <c r="C4">
-        <v>100</v>
-      </c>
-      <c r="D4">
-        <v>4</v>
-      </c>
-      <c r="E4">
-        <f>D4*$C$1</f>
-        <v>64</v>
-      </c>
-      <c r="F4" s="6">
-        <f>_xlfn.CEILING.MATH((E4)/C4)</f>
-        <v>1</v>
-      </c>
-      <c r="G4" s="2">
-        <v>9.8699999999999992</v>
-      </c>
-      <c r="H4" s="4">
-        <f>F4*G4</f>
-        <v>9.8699999999999992</v>
-      </c>
-      <c r="I4" s="4">
-        <f>H4/E4</f>
-        <v>0.15421874999999999</v>
-      </c>
-      <c r="J4" t="s">
-        <v>23</v>
-      </c>
-      <c r="K4" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" t="s">
-        <v>72</v>
-      </c>
-      <c r="C5">
-        <v>50</v>
-      </c>
-      <c r="D5">
-        <v>8</v>
-      </c>
-      <c r="E5">
-        <f t="shared" ref="E5:E14" si="0">D5*$C$1</f>
-        <v>128</v>
-      </c>
-      <c r="F5" s="6">
-        <f t="shared" ref="F5:F14" si="1">_xlfn.CEILING.MATH((D5*$C$1)/C5)</f>
-        <v>3</v>
-      </c>
-      <c r="G5" s="2">
-        <v>8.64</v>
-      </c>
-      <c r="H5" s="4">
-        <f t="shared" ref="H5:H14" si="2">F5*G5</f>
-        <v>25.92</v>
-      </c>
-      <c r="I5" s="4">
-        <f t="shared" ref="I5:I14" si="3">H5/E5</f>
-        <v>0.20250000000000001</v>
-      </c>
-      <c r="J5" t="s">
-        <v>24</v>
-      </c>
-      <c r="K5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6">
-        <v>50</v>
-      </c>
-      <c r="D6">
-        <v>12</v>
-      </c>
-      <c r="E6">
-        <f t="shared" si="0"/>
-        <v>192</v>
-      </c>
-      <c r="F6" s="6">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="G6" s="2">
-        <v>12.53</v>
-      </c>
-      <c r="H6" s="4">
-        <f t="shared" si="2"/>
-        <v>50.12</v>
-      </c>
-      <c r="I6" s="4">
-        <f t="shared" si="3"/>
-        <v>0.26104166666666667</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-      <c r="K6" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>70</v>
-      </c>
-      <c r="C7">
-        <v>50</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-      <c r="F7" s="6">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G7" s="2">
-        <v>5.72</v>
-      </c>
-      <c r="H7" s="4">
-        <f t="shared" si="2"/>
-        <v>11.44</v>
-      </c>
-      <c r="I7" s="4">
-        <f t="shared" si="3"/>
-        <v>0.17874999999999999</v>
-      </c>
-      <c r="J7" t="s">
-        <v>71</v>
-      </c>
-      <c r="K7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8">
-        <v>100</v>
-      </c>
-      <c r="D8">
-        <v>6</v>
-      </c>
-      <c r="E8">
-        <f t="shared" si="0"/>
-        <v>96</v>
-      </c>
-      <c r="F8" s="6">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="G8" s="2">
-        <v>7.46</v>
-      </c>
-      <c r="H8" s="4">
-        <f t="shared" si="2"/>
-        <v>7.46</v>
-      </c>
-      <c r="I8" s="4">
-        <f t="shared" si="3"/>
-        <v>7.7708333333333338E-2</v>
-      </c>
-      <c r="J8" t="s">
-        <v>26</v>
-      </c>
-      <c r="K8" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9">
-        <v>25</v>
-      </c>
-      <c r="D9">
-        <v>2</v>
-      </c>
-      <c r="E9">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="F9" s="6">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G9" s="2">
-        <v>5.2</v>
-      </c>
-      <c r="H9" s="4">
-        <f t="shared" si="2"/>
-        <v>10.4</v>
-      </c>
-      <c r="I9" s="4">
-        <f t="shared" si="3"/>
-        <v>0.32500000000000001</v>
-      </c>
-      <c r="J9" t="s">
-        <v>27</v>
-      </c>
-      <c r="K9" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" t="s">
-        <v>16</v>
-      </c>
-      <c r="C10">
-        <v>100</v>
-      </c>
-      <c r="D10">
-        <v>16</v>
-      </c>
-      <c r="E10">
-        <f t="shared" si="0"/>
-        <v>256</v>
-      </c>
-      <c r="F10" s="6">
-        <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-      <c r="G10" s="2">
-        <v>8.77</v>
-      </c>
-      <c r="H10" s="4">
-        <f t="shared" si="2"/>
-        <v>26.31</v>
-      </c>
-      <c r="I10" s="4">
-        <f t="shared" si="3"/>
-        <v>0.1027734375</v>
-      </c>
-      <c r="J10" t="s">
-        <v>28</v>
-      </c>
-      <c r="K10" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" t="s">
-        <v>18</v>
-      </c>
-      <c r="C11">
-        <v>50</v>
-      </c>
-      <c r="D11">
-        <v>2</v>
-      </c>
-      <c r="E11">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="F11" s="6">
-        <f t="shared" si="1"/>
-        <v>1</v>
-      </c>
-      <c r="G11" s="2">
-        <v>10.44</v>
-      </c>
-      <c r="H11" s="4">
-        <f t="shared" si="2"/>
-        <v>10.44</v>
-      </c>
-      <c r="I11" s="4">
-        <f t="shared" si="3"/>
-        <v>0.32624999999999998</v>
-      </c>
-      <c r="J11" t="s">
-        <v>29</v>
-      </c>
-      <c r="K11" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12">
-        <v>10</v>
-      </c>
-      <c r="D12">
-        <v>2</v>
-      </c>
-      <c r="E12">
-        <f t="shared" si="0"/>
-        <v>32</v>
-      </c>
-      <c r="F12" s="6">
-        <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-      <c r="G12" s="2">
-        <v>7</v>
-      </c>
-      <c r="H12" s="4">
-        <f t="shared" si="2"/>
-        <v>28</v>
-      </c>
-      <c r="I12" s="4">
-        <f t="shared" si="3"/>
-        <v>0.875</v>
-      </c>
-      <c r="J12" t="s">
-        <v>31</v>
-      </c>
-      <c r="K12" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
-        <v>33</v>
-      </c>
-      <c r="B13" t="s">
-        <v>34</v>
-      </c>
-      <c r="C13">
-        <v>1</v>
-      </c>
-      <c r="D13">
-        <v>1</v>
-      </c>
-      <c r="E13">
-        <f t="shared" si="0"/>
-        <v>16</v>
-      </c>
-      <c r="F13" s="6">
-        <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-      <c r="G13" s="2">
-        <v>4.7</v>
-      </c>
-      <c r="H13" s="4">
-        <f t="shared" si="2"/>
-        <v>75.2</v>
-      </c>
-      <c r="I13" s="4">
-        <f t="shared" si="3"/>
-        <v>4.7</v>
-      </c>
-      <c r="J13" t="s">
-        <v>35</v>
-      </c>
-      <c r="K13" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14">
-        <v>50</v>
-      </c>
-      <c r="D14">
-        <v>4</v>
-      </c>
-      <c r="E14">
-        <f t="shared" si="0"/>
-        <v>64</v>
-      </c>
-      <c r="F14" s="6">
-        <f t="shared" si="1"/>
-        <v>2</v>
-      </c>
-      <c r="G14" s="2">
-        <v>9.4</v>
-      </c>
-      <c r="H14" s="4">
-        <f t="shared" si="2"/>
-        <v>18.8</v>
-      </c>
-      <c r="I14" s="4">
-        <f t="shared" si="3"/>
-        <v>0.29375000000000001</v>
-      </c>
-      <c r="J14" t="s">
-        <v>49</v>
-      </c>
-      <c r="K14" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="G16" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="H16" s="4">
-        <f>SUM(H4:H14)</f>
-        <v>273.95999999999998</v>
-      </c>
-    </row>
-    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
-      <c r="G17" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H17" s="4">
-        <f>H16/C1</f>
-        <v>17.122499999999999</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8A2C5A5-03CA-4DB8-9D15-15879A9BBD02}">
   <dimension ref="A1:H15"/>
   <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
@@ -1580,4 +1131,667 @@
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{421C52AF-D934-5E4D-A590-21C8983DA813}">
+  <dimension ref="A1:K17"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="11.69921875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.796875" style="6"/>
+    <col min="7" max="7" width="13.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="59.296875" customWidth="1"/>
+    <col min="11" max="11" width="38.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C4">
+        <v>100</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <f>D4*$C$1</f>
+        <v>64</v>
+      </c>
+      <c r="F4" s="6">
+        <f>_xlfn.CEILING.MATH((E4)/C4)</f>
+        <v>1</v>
+      </c>
+      <c r="G4" s="2">
+        <v>9.8699999999999992</v>
+      </c>
+      <c r="H4" s="4">
+        <f>F4*G4</f>
+        <v>9.8699999999999992</v>
+      </c>
+      <c r="I4" s="4">
+        <f>H4/E4</f>
+        <v>0.15421874999999999</v>
+      </c>
+      <c r="J4" t="s">
+        <v>23</v>
+      </c>
+      <c r="K4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5">
+        <v>50</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
+        <f t="shared" ref="E5:E14" si="0">D5*$C$1</f>
+        <v>128</v>
+      </c>
+      <c r="F5" s="6">
+        <f t="shared" ref="F5:F14" si="1">_xlfn.CEILING.MATH((D5*$C$1)/C5)</f>
+        <v>3</v>
+      </c>
+      <c r="G5" s="2">
+        <v>8.64</v>
+      </c>
+      <c r="H5" s="4">
+        <f t="shared" ref="H5:H14" si="2">F5*G5</f>
+        <v>25.92</v>
+      </c>
+      <c r="I5" s="4">
+        <f t="shared" ref="I5:I14" si="3">H5/E5</f>
+        <v>0.20250000000000001</v>
+      </c>
+      <c r="J5" t="s">
+        <v>24</v>
+      </c>
+      <c r="K5" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6">
+        <v>50</v>
+      </c>
+      <c r="D6">
+        <v>12</v>
+      </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>192</v>
+      </c>
+      <c r="F6" s="6">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G6" s="2">
+        <v>12.53</v>
+      </c>
+      <c r="H6" s="4">
+        <f t="shared" si="2"/>
+        <v>50.12</v>
+      </c>
+      <c r="I6" s="4">
+        <f t="shared" si="3"/>
+        <v>0.26104166666666667</v>
+      </c>
+      <c r="J6" t="s">
+        <v>25</v>
+      </c>
+      <c r="K6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C7">
+        <v>50</v>
+      </c>
+      <c r="D7">
+        <v>4</v>
+      </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="F7" s="6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G7" s="2">
+        <v>5.72</v>
+      </c>
+      <c r="H7" s="4">
+        <f t="shared" si="2"/>
+        <v>11.44</v>
+      </c>
+      <c r="I7" s="4">
+        <f t="shared" si="3"/>
+        <v>0.17874999999999999</v>
+      </c>
+      <c r="J7" t="s">
+        <v>71</v>
+      </c>
+      <c r="K7" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8">
+        <v>100</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>96</v>
+      </c>
+      <c r="F8" s="6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G8" s="2">
+        <v>7.46</v>
+      </c>
+      <c r="H8" s="4">
+        <f t="shared" si="2"/>
+        <v>7.46</v>
+      </c>
+      <c r="I8" s="4">
+        <f t="shared" si="3"/>
+        <v>7.7708333333333338E-2</v>
+      </c>
+      <c r="J8" t="s">
+        <v>26</v>
+      </c>
+      <c r="K8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9">
+        <v>25</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="F9" s="6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>5.2</v>
+      </c>
+      <c r="H9" s="4">
+        <f t="shared" si="2"/>
+        <v>10.4</v>
+      </c>
+      <c r="I9" s="4">
+        <f t="shared" si="3"/>
+        <v>0.32500000000000001</v>
+      </c>
+      <c r="J9" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>15</v>
+      </c>
+      <c r="B10" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10">
+        <v>100</v>
+      </c>
+      <c r="D10">
+        <v>16</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>256</v>
+      </c>
+      <c r="F10" s="6">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="G10" s="2">
+        <v>8.77</v>
+      </c>
+      <c r="H10" s="4">
+        <f t="shared" si="2"/>
+        <v>26.31</v>
+      </c>
+      <c r="I10" s="4">
+        <f t="shared" si="3"/>
+        <v>0.1027734375</v>
+      </c>
+      <c r="J10" t="s">
+        <v>28</v>
+      </c>
+      <c r="K10" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11">
+        <v>50</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="F11" s="6">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="G11" s="2">
+        <v>10.44</v>
+      </c>
+      <c r="H11" s="4">
+        <f t="shared" si="2"/>
+        <v>10.44</v>
+      </c>
+      <c r="I11" s="4">
+        <f t="shared" si="3"/>
+        <v>0.32624999999999998</v>
+      </c>
+      <c r="J11" t="s">
+        <v>29</v>
+      </c>
+      <c r="K11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12">
+        <v>10</v>
+      </c>
+      <c r="D12">
+        <v>2</v>
+      </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>32</v>
+      </c>
+      <c r="F12" s="6">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="G12" s="2">
+        <v>7</v>
+      </c>
+      <c r="H12" s="4">
+        <f t="shared" si="2"/>
+        <v>28</v>
+      </c>
+      <c r="I12" s="4">
+        <f t="shared" si="3"/>
+        <v>0.875</v>
+      </c>
+      <c r="J12" t="s">
+        <v>31</v>
+      </c>
+      <c r="K12" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="B13" t="s">
+        <v>34</v>
+      </c>
+      <c r="C13">
+        <v>1</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="F13" s="6">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="G13" s="2">
+        <v>4.7</v>
+      </c>
+      <c r="H13" s="4">
+        <f t="shared" si="2"/>
+        <v>75.2</v>
+      </c>
+      <c r="I13" s="4">
+        <f t="shared" si="3"/>
+        <v>4.7</v>
+      </c>
+      <c r="J13" t="s">
+        <v>35</v>
+      </c>
+      <c r="K13" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>48</v>
+      </c>
+      <c r="C14">
+        <v>50</v>
+      </c>
+      <c r="D14">
+        <v>4</v>
+      </c>
+      <c r="E14">
+        <f t="shared" si="0"/>
+        <v>64</v>
+      </c>
+      <c r="F14" s="6">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="G14" s="2">
+        <v>9.4</v>
+      </c>
+      <c r="H14" s="4">
+        <f t="shared" si="2"/>
+        <v>18.8</v>
+      </c>
+      <c r="I14" s="4">
+        <f t="shared" si="3"/>
+        <v>0.29375000000000001</v>
+      </c>
+      <c r="J14" t="s">
+        <v>49</v>
+      </c>
+      <c r="K14" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="G16" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="H16" s="4">
+        <f>SUM(H4:H14)</f>
+        <v>273.95999999999998</v>
+      </c>
+    </row>
+    <row r="17" spans="7:8" x14ac:dyDescent="0.3">
+      <c r="G17" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="H17" s="4">
+        <f>H16/C1</f>
+        <v>17.122499999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{93DE9E05-E823-43C4-A861-DE9DC42986E3}">
+  <dimension ref="A1:H8"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="19.69921875" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" style="16" customWidth="1"/>
+    <col min="5" max="5" width="10" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.09765625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="41.796875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.69921875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C2">
+        <v>2</v>
+      </c>
+      <c r="D2" s="16">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2">
+        <v>20</v>
+      </c>
+      <c r="F2" s="4">
+        <f>E2*C2</f>
+        <v>40</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" s="16">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>11.5</v>
+      </c>
+      <c r="F3" s="4">
+        <f>E3*C3</f>
+        <v>11.5</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C4">
+        <v>4</v>
+      </c>
+      <c r="D4" s="16">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2">
+        <v>24</v>
+      </c>
+      <c r="F4" s="4">
+        <f>E4*C4</f>
+        <v>96</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="H4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
+      </c>
+      <c r="D5" s="16">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2">
+        <v>41</v>
+      </c>
+      <c r="F5" s="4">
+        <f>E5*C5</f>
+        <v>82</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="H5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="E8" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="F8" s="4">
+        <f>SUM(F2:F6)</f>
+        <v>229.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G2" r:id="rId1" xr:uid="{8239E42D-FB55-414F-805E-F9561B0EEA2B}"/>
+    <hyperlink ref="G3" r:id="rId2" xr:uid="{BE1B5B5A-D7D2-49D0-BD62-CA56A155B200}"/>
+    <hyperlink ref="G4" r:id="rId3" xr:uid="{051E9697-156E-412C-B499-51F967165E84}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{F7578765-BAAD-44AF-B3D9-42D048226111}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>